<commit_message>
docs: add execution proof screenshots with sensitive data redacted
</commit_message>
<xml_diff>
--- a/examples/sample_data.xlsx
+++ b/examples/sample_data.xlsx
@@ -539,7 +539,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PUSKESMAS SERPONG II — DINAS KESEHATAN KOTA TANGERANG SELATAN</t>
+          <t>PUSKESMAS CONTOH — DINAS KESEHATAN KABUPATEN/KOTA</t>
         </is>
       </c>
     </row>
@@ -553,7 +553,7 @@
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Dicetak: 16 June 2026    |    Sumber: SIMPUS Web Kemkes RI    |    ⚠ File ini berisi DATA DUMMY — aman untuk demo dan pengujian</t>
+          <t>Dicetak: 22 October 2026    |    Sumber: SIMPUS Web Kemkes RI    |    ⚠ File ini berisi DATA DUMMY — aman untuk demo dan pengujian</t>
         </is>
       </c>
     </row>

</xml_diff>